<commit_message>
Entity graph scoring: a second score out of 100 for the schema graph, on every page and every report
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FeWbztza33MhFGyQMY13SN
</commit_message>
<xml_diff>
--- a/seo-audit-pages.xlsx
+++ b/seo-audit-pages.xlsx
@@ -9,26 +9,30 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every page" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Moves" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI answers" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitors" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlinks" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site checks" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redirects" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entity graph" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema types" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Moves" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI answers" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitors" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlinks" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site checks" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redirects" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Every page'!$A$1:$AE$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Every page'!$A$1:$AI$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings'!$A$1:$F$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Moves'!$A$1:$E$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Opportunities'!$A$1:$E$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Questions'!$A$1:$C$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'AI answers'!$A$1:$L$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Competitors'!$A$1:$D$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backlinks'!$A$1:$D$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Site checks'!$A$1:$B$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Redirects'!$A$1:$D$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Entity graph'!$A$1:$F$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Schema types'!$A$1:$C$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Moves'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Opportunities'!$A$1:$E$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Questions'!$A$1:$C$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'AI answers'!$A$1:$L$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Competitors'!$A$1:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Backlinks'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Site checks'!$A$1:$B$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Redirects'!$A$1:$D$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE27"/>
+  <dimension ref="A1:AI27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -488,9 +492,13 @@
     <col width="40" customWidth="1" min="26" max="26"/>
     <col width="8" customWidth="1" min="27" max="27"/>
     <col width="8" customWidth="1" min="28" max="28"/>
-    <col width="90" customWidth="1" min="29" max="29"/>
-    <col width="36" customWidth="1" min="30" max="30"/>
-    <col width="10" customWidth="1" min="31" max="31"/>
+    <col width="8" customWidth="1" min="29" max="29"/>
+    <col width="7" customWidth="1" min="30" max="30"/>
+    <col width="8" customWidth="1" min="31" max="31"/>
+    <col width="34" customWidth="1" min="32" max="32"/>
+    <col width="90" customWidth="1" min="33" max="33"/>
+    <col width="36" customWidth="1" min="34" max="34"/>
+    <col width="10" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -636,15 +644,35 @@
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
+          <t>Entity score</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Entity grade</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Schema nodes</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Entity checks failing</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
           <t>What we would do</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>New path in the build</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
@@ -765,17 +793,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Give the page exactly one H1; Break the copy into two or more H2 sections; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC2" t="n">
+        <v>71</v>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AE2" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>person, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Give the page exactly one H1; Break the copy into two or more H2 sections; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Name the expert or author as a Person, with a URL that identifies them; Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
           <t>/about.html</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -896,17 +940,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Give the page exactly one H1; Break the copy into two or more H2 sections; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC3" t="n">
+        <v>71</v>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AE3" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>person, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Give the page exactly one H1; Break the copy into two or more H2 sections; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Name the expert or author as a Person, with a URL that identifies them; Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
           <t>/about.html</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr">
+      <c r="AI3" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -1027,17 +1087,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Give the page exactly one H1; Break the copy into two or more H2 sections; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC4" t="n">
+        <v>71</v>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AE4" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>person, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Give the page exactly one H1; Break the copy into two or more H2 sections; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Name the expert or author as a Person, with a URL that identifies them; Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
           <t>/about.html</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AI4" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -1162,17 +1238,33 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Break the copy into two or more H2 sections; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image)</t>
-        </is>
+      <c r="AC5" t="n">
+        <v>66</v>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AE5" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>person, area, contact, about, clean</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Break the copy into two or more H2 sections; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Name the expert or author as a Person, with a URL that identifies them; Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType; Remove empty and placeholder values from the markup</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
           <t>/contact.html</t>
         </is>
       </c>
-      <c r="AE5" t="inlineStr">
+      <c r="AI5" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -1264,7 +1356,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -1297,17 +1389,33 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image)</t>
-        </is>
+      <c r="AC6" t="n">
+        <v>45</v>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE6" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
           <t>/contact.html</t>
         </is>
       </c>
-      <c r="AE6" t="inlineStr">
+      <c r="AI6" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -1432,17 +1540,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC7" t="n">
+        <v>71</v>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AE7" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>person, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Name the expert or author as a Person, with a URL that identifies them; Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
           <t>/industries.html</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr">
+      <c r="AI7" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -1534,7 +1658,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1567,17 +1691,33 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image)</t>
-        </is>
+      <c r="AC8" t="n">
+        <v>45</v>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE8" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
           <t>/contact.html</t>
         </is>
       </c>
-      <c r="AE8" t="inlineStr">
+      <c r="AI8" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -1669,7 +1809,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1702,17 +1842,33 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image)</t>
-        </is>
+      <c r="AC9" t="n">
+        <v>45</v>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE9" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
           <t>/contact.html</t>
         </is>
       </c>
-      <c r="AE9" t="inlineStr">
+      <c r="AI9" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -1804,7 +1960,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1837,17 +1993,33 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image)</t>
-        </is>
+      <c r="AC10" t="n">
+        <v>45</v>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE10" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
           <t>/contact.html</t>
         </is>
       </c>
-      <c r="AE10" t="inlineStr">
+      <c r="AI10" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -1972,17 +2144,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Alt text on every image; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC11" t="n">
+        <v>71</v>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AE11" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>person, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Alt text on every image; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Name the expert or author as a Person, with a URL that identifies them; Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
           <t>/services/cybersecurity.html</t>
         </is>
       </c>
-      <c r="AE11" t="inlineStr">
+      <c r="AI11" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -2107,17 +2295,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC12" t="n">
+        <v>71</v>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AE12" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>person, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Name the expert or author as a Person, with a URL that identifies them; Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
           <t>/about.html</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr">
+      <c r="AI12" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -2242,17 +2446,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC13" t="n">
+        <v>71</v>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AE13" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>person, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Name the expert or author as a Person, with a URL that identifies them; Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
           <t>/about.html</t>
         </is>
       </c>
-      <c r="AE13" t="inlineStr">
+      <c r="AI13" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -2344,7 +2564,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -2377,17 +2597,33 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AC14" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image)</t>
-        </is>
+      <c r="AC14" t="n">
+        <v>45</v>
       </c>
       <c r="AD14" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE14" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Add a heading that asks the question the page answers; Deepen to 300 words or more; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
           <t>/contact.html</t>
         </is>
       </c>
-      <c r="AE14" t="inlineStr">
+      <c r="AI14" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -2512,17 +2748,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC15" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC15" t="n">
+        <v>48</v>
       </c>
       <c r="AD15" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE15" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
           <t>/industries/life-sciences.html</t>
         </is>
       </c>
-      <c r="AE15" t="inlineStr">
+      <c r="AI15" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -2614,7 +2866,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
@@ -2647,17 +2899,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC16" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC16" t="n">
+        <v>48</v>
       </c>
       <c r="AD16" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE16" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
           <t>/services/managed-it.html</t>
         </is>
       </c>
-      <c r="AE16" t="inlineStr">
+      <c r="AI16" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -2749,7 +3017,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
@@ -2782,17 +3050,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC17" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC17" t="n">
+        <v>48</v>
       </c>
       <c r="AD17" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE17" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
           <t>/services/site-intelligence.html</t>
         </is>
       </c>
-      <c r="AE17" t="inlineStr">
+      <c r="AI17" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -2884,7 +3168,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
@@ -2917,17 +3201,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC18" t="inlineStr">
-        <is>
-          <t>Rewrite the title to 30 to 60 characters; Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC18" t="n">
+        <v>74</v>
       </c>
       <c r="AD18" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AE18" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>person, area, contact, clean</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>Rewrite the title to 30 to 60 characters; Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Name the expert or author as a Person, with a URL that identifies them; Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Remove empty and placeholder values from the markup</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
           <t>/index.html</t>
         </is>
       </c>
-      <c r="AE18" t="inlineStr">
+      <c r="AI18" t="inlineStr">
         <is>
           <t>merged</t>
         </is>
@@ -3048,17 +3348,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC19" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Break the copy into two or more H2 sections; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC19" t="n">
+        <v>71</v>
       </c>
       <c r="AD19" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AE19" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>person, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Break the copy into two or more H2 sections; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Name the expert or author as a Person, with a URL that identifies them; Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
           <t>/voices.html</t>
         </is>
       </c>
-      <c r="AE19" t="inlineStr">
+      <c r="AI19" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -3150,7 +3466,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
@@ -3183,17 +3499,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC20" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Alt text on every image; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC20" t="n">
+        <v>71</v>
       </c>
       <c r="AD20" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AE20" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>person, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Alt text on every image; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Name the expert or author as a Person, with a URL that identifies them; Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
           <t>/why-nexus.html</t>
         </is>
       </c>
-      <c r="AE20" t="inlineStr">
+      <c r="AI20" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -3318,17 +3650,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC21" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Alt text on every image; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC21" t="n">
+        <v>48</v>
       </c>
       <c r="AD21" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE21" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Alt text on every image; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
           <t>/industries/growing-businesses.html</t>
         </is>
       </c>
-      <c r="AE21" t="inlineStr">
+      <c r="AI21" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -3453,17 +3801,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC22" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC22" t="n">
+        <v>48</v>
       </c>
       <c r="AD22" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE22" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
           <t>/industries/manufacturing.html</t>
         </is>
       </c>
-      <c r="AE22" t="inlineStr">
+      <c r="AI22" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -3588,17 +3952,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC23" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC23" t="n">
+        <v>48</v>
       </c>
       <c r="AD23" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE23" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
           <t>/industries/professional-services.html</t>
         </is>
       </c>
-      <c r="AE23" t="inlineStr">
+      <c r="AI23" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -3690,7 +4070,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
@@ -3723,17 +4103,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC24" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC24" t="n">
+        <v>48</v>
       </c>
       <c r="AD24" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Add a heading that asks the question the page answers; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
           <t>/services/consultation-projects.html</t>
         </is>
       </c>
-      <c r="AE24" t="inlineStr">
+      <c r="AI24" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -3825,7 +4221,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
@@ -3858,17 +4254,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC25" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC25" t="n">
+        <v>48</v>
       </c>
       <c r="AD25" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE25" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Write a meta description of 70 to 160 characters; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
           <t>/services/networking.html</t>
         </is>
       </c>
-      <c r="AE25" t="inlineStr">
+      <c r="AI25" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -3956,7 +4368,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
@@ -3989,17 +4401,33 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC26" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Alt text on every image; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC26" t="n">
+        <v>48</v>
       </c>
       <c r="AD26" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE26" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Alt text on every image; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
           <t>/services.html</t>
         </is>
       </c>
-      <c r="AE26" t="inlineStr">
+      <c r="AI26" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
@@ -4091,7 +4519,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
@@ -4124,29 +4552,537 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AC27" t="inlineStr">
-        <is>
-          <t>Add the city or service area to the title; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page</t>
-        </is>
+      <c r="AC27" t="n">
+        <v>48</v>
       </c>
       <c r="AD27" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AE27" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>primary, provider, area, contact, about</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>Add the city or service area to the title; Add a five-question FAQ marked up as FAQPage; Add Service schema (or Article schema on a post); Add LocalBusiness schema with the office address; Add Review or AggregateRating schema from real Google reviews; Set a branded share image (og:image); Put a form or a tap-to-call number on the page; Add the entity this page is about (Service, LocalBusiness, Article or Product); Link this page's entity to the Organization (provider, publisher or parentOrganization); Add areaServed or a postal address to the entity; Add contactPoint or a telephone to the Organization; Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
           <t>/services/meeting-spaces.html</t>
         </is>
       </c>
-      <c r="AE27" t="inlineStr">
+      <c r="AI27" t="inlineStr">
         <is>
           <t>rebuilt</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AE27"/>
+  <autoFilter ref="A1:AI27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Authority Score</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Referring domains</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Backlinks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>nexusnt.com</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>316</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>managedits.com</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1,199</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>computerbilities.com</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>561</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2,987</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>worksmart.com</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>819</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3,945</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>scarlettgroup.com</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>48,512</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="70" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>nexusnt.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>sitemap_urls</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>http_redirects_to_https</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>one_canonical_host</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>canonical_host</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>www.nexusnt.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>robots_status</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>allows_gptbot</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>allows_claudebot</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>allows_perplexitybot</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>allows_google-extended</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>allows_bingbot</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>allows_googlebot</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>sitemap_declared</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>llms_txt</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Served over HTTPS with one canonical host (www)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>robots.txt allows Google and all four AI crawlers (GPTBot, ClaudeBot, PerplexityBot, Google-Extended)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sitemap declared, 26 URLs</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Organization schema on every page (Yoast)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LocalBusiness schema for the Morrisville office</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>FAQPage schema anywhere on the site</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Service schema on any service page</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Address, phone or sameAs in the Organization schema</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>A share image (og:image) on any page</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>A blog, guide or any page that answers a question</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>llms.txt published for AI assistants</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Forms create CRM records (custom step forms today)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B27"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5160,6 +6096,664 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Pages carrying it</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Pages it applies to</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A named Person, not a byline string</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Name the expert or author as a Person, with a URL that identifies them</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>areaServed or a postal address</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Add areaServed or a postal address to the entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>author linked to a Person</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Point author at a Person object, not a plain string</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>contactPoint or telephone</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>26</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Add contactPoint or a telephone to the Organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>about, mentions or serviceType naming the topic</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>21</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Name what the page is about with about, mentions or serviceType</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Primary entity for this kind of page</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>11</v>
+      </c>
+      <c r="C7" t="n">
+        <v>26</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>42%</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>14</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Add the entity this page is about (Service, LocalBusiness, Article or Product)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Primary entity linked to the Organization</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" t="n">
+        <v>26</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>42%</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Link this page's entity to the Organization (provider, publisher or parentOrganization)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>No empty or placeholder values</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C9" t="n">
+        <v>26</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Remove empty and placeholder values from the markup</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Organization identified</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>26</v>
+      </c>
+      <c r="C10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Add Organization schema naming the company</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Page type declared</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>26</v>
+      </c>
+      <c r="C11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Declare the page type (WebPage, Article, CollectionPage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WebSite on the home page</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Add WebSite schema on the home page</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BreadcrumbList</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>20</v>
+      </c>
+      <c r="C13" t="n">
+        <v>20</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Add BreadcrumbList so the hierarchy is machine-readable</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>sameAs to authoritative profiles</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>26</v>
+      </c>
+      <c r="C14" t="n">
+        <v>26</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Add sameAs to the company's LinkedIn, Google Business Profile and other authoritative profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>datePublished and dateModified</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>21</v>
+      </c>
+      <c r="C15" t="n">
+        <v>21</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Add datePublished and dateModified</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>@id on the main entities</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>26</v>
+      </c>
+      <c r="C16" t="n">
+        <v>26</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Give the main entities a stable @id so they can be referenced</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Every @id reference resolves</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>26</v>
+      </c>
+      <c r="C17" t="n">
+        <v>26</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Point every @id reference at an entity that exists</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F17"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Pages</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share of the site</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WebPage</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>26</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Organization</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>26</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PropertyValueSpecification</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>26</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ListItem</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>26</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BreadcrumbList</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>26</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SearchAction</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>26</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EntryPoint</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>26</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ImageObject</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>26</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ReadAction</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>26</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WebSite</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>26</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5328,7 +6922,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5809,7 +7403,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6203,7 +7797,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6788,7 +8382,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6983,496 +8577,4 @@
   <autoFilter ref="A1:D8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Domain</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Authority Score</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Referring domains</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Backlinks</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>nexusnt.com</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>180</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>316</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>managedits.com</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>256</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1,199</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>computerbilities.com</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>561</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2,987</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>worksmart.com</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>819</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>3,945</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>scarlettgroup.com</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>902</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>48,512</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:D6"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="70" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>domain</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>nexusnt.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>sitemap_urls</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>http_redirects_to_https</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>one_canonical_host</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>canonical_host</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>www.nexusnt.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>robots_status</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>allows_gptbot</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>allows_claudebot</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>allows_perplexitybot</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>allows_google-extended</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>allows_bingbot</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>allows_googlebot</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>sitemap_declared</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>llms_txt</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Served over HTTPS with one canonical host (www)</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>robots.txt allows Google and all four AI crawlers (GPTBot, ClaudeBot, PerplexityBot, Google-Extended)</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Sitemap declared, 26 URLs</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Organization schema on every page (Yoast)</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>LocalBusiness schema for the Morrisville office</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>FAQPage schema anywhere on the site</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Service schema on any service page</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Address, phone or sameAs in the Organization schema</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>A share image (og:image) on any page</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>A blog, guide or any page that answers a question</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>llms.txt published for AI assistants</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Forms create CRM records (custom step forms today)</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B27"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>